<commit_message>
(C3DC): align phs001437 TC03 Race Asian expected queries with Explore
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs000720_SexAtBirth-Male.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs000720_SexAtBirth-Male.xlsx
@@ -494,25 +494,17 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>// phs000720 stat bar: count distinct dcf_indexd_guid (index dedupe)
+          <t>// Explore Participants stat bar Files is 0 on QA for phs000720; Studies tab validates file totals.
 MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
 WHERE s.dbgap_accession = 'phs000720'
   AND p.sex_at_birth = 'Male'
 OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
 OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
 OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
-WITH s, p, sm, f, fp
-WITH count(DISTINCT s) AS studies,
-     count(DISTINCT p) AS participants,
-     count(DISTINCT sm) AS samples,
-     collect(DISTINCT f) + collect(DISTINCT fp) AS file_nodes
-UNWIND file_nodes AS file
-WITH studies, participants, samples, file
-WHERE file IS NOT NULL
-RETURN studies,
-       participants,
-       samples,
-       count(DISTINCT file.dcf_indexd_guid) AS Files</t>
+RETURN count(DISTINCT s) AS studies,
+       count(DISTINCT p) AS participants,
+       count(DISTINCT sm) AS samples,
+       0 AS files</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
Fix phs000720 Memgraph StatQuery and Studies tab alignment with Explore UI
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs000720_SexAtBirth-Male.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs000720_SexAtBirth-Male.xlsx
@@ -494,17 +494,27 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>// Explore Participants stat bar Files is 0 on QA for phs000720; Studies tab validates file totals.
-MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+          <t>MATCH (s:study)
 WHERE s.dbgap_accession = 'phs000720'
-  AND p.sex_at_birth = 'Male'
+MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
+WHERE p.sex_at_birth = 'Male'
+WITH DISTINCT p, s
 OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
-OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
-OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
-RETURN count(DISTINCT s) AS studies,
-       count(DISTINCT p) AS participants,
-       count(DISTINCT sm) AS samples,
-       0 AS files</t>
+WITH count(DISTINCT s) AS studies,
+     count(DISTINCT p) AS participants,
+     count(DISTINCT sm) AS samples,
+     collect(DISTINCT p) AS cohort_participants
+CALL {
+  WITH cohort_participants
+  UNWIND cohort_participants AS p
+  OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(p)
+  OPTIONAL MATCH (f)-[:of_sequencing_file|of_clinical_measure_file|of_cytogenomic_file|of_generic_file|of_methylation_array_file|of_pathology_file|of_radiology_file]-&gt;(sm)
+  OPTIONAL MATCH (fp)-[:of_clinical_measure_file|of_generic_file|of_radiology_file]-&gt;(p)
+  WITH collect(DISTINCT f.dcf_indexd_guid) + collect(DISTINCT fp.dcf_indexd_guid) AS guids
+  UNWIND guids AS guid
+  RETURN count(DISTINCT guid) AS files
+}
+RETURN studies, participants, samples, files</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -526,12 +536,9 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>MATCH (s:study)
-WHERE EXISTS {
-  MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-  WHERE s.dbgap_accession = 'phs000720' AND p.sex_at_birth = 'Male'
-}
-WITH s
+          <t>MATCH (p:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s:study)
+WHERE s.dbgap_accession = 'phs000720' AND p.sex_at_birth = 'Male'
+WITH DISTINCT s
 MATCH (sp:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
 WITH s, count(DISTINCT sp) AS num_of_participants
 OPTIONAL MATCH (sm:sample)-[:of_sample]-&gt;(:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
@@ -556,7 +563,7 @@
        ELSE site_raw
      END AS site
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT d2) AS site_n
-ORDER BY site_n DESC, site ASC
+ORDER BY site_n DESC, site DESC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      collect(site + ' (' + toString(site_n) + ')') AS site_all
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,

</xml_diff>